<commit_message>
Anomalies SF1-RPS4 — 25/09/2026
</commit_message>
<xml_diff>
--- a/presentation/SF1-RPS4/anomalies.xlsx
+++ b/presentation/SF1-RPS4/anomalies.xlsx
@@ -17,17 +17,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
-  </numFmts>
-  <fonts count="2">
+  <numFmts count="0"/>
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -48,7 +48,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -56,16 +56,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -431,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U7"/>
+  <dimension ref="A1:T1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -451,10 +456,9 @@
     <col width="13" customWidth="1" min="15" max="15"/>
     <col width="27" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="16" customWidth="1" min="18" max="18"/>
-    <col width="12" customWidth="1" min="19" max="19"/>
-    <col width="15" customWidth="1" min="20" max="20"/>
-    <col width="22" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="15" customWidth="1" min="19" max="19"/>
+    <col width="22" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -545,532 +549,17 @@
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>Nb anomalies</t>
+          <t>Anomalie</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>Anomalie</t>
+          <t>Responsable</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>Responsable</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
           <t>Action recommandée</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>12873728</v>
-      </c>
-      <c r="B2" t="n">
-        <v>4002050621</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Tirage de câble pour installation caméra</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>OR004002050621</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>SF01-PS-PS04-SECGAZ-0F8302-CSUR</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>CONTRÔLE ET SURVEILLANCE</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>SF1-RPS4</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>GM0</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>SF01</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>LANC CCRP PART RIMP</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>SOPL</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>MOUSSAHIF</t>
-        </is>
-      </c>
-      <c r="P2" s="2" t="n">
-        <v>46216</v>
-      </c>
-      <c r="Q2" s="2" t="n">
-        <v>46178</v>
-      </c>
-      <c r="R2" t="n">
-        <v>2</v>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>TAUX_REALISATION_CORRECTIF/PT | OT exécution 1mois&lt; &lt;3mois</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>Chef d'atelier</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>Ameliorer le taux de realisation des OT correctifs. | Reduire les OT en execution entre 1 et 3 mois.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>13179459</v>
-      </c>
-      <c r="B3" t="n">
-        <v>4002317916</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>chasse des filtres d'eau de mer  hors se</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>OR004002317916</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>SF01-PS-PS04-SECACI</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>SECTION ACIDE DE L'ATELIER PS 4</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>SF1-RPS4</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>GM4</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>SF01</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>LANC CCRP PART RIMP</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>SOPL</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>BENMOUSSA1</t>
-        </is>
-      </c>
-      <c r="P3" s="2" t="n">
-        <v>46223</v>
-      </c>
-      <c r="Q3" s="2" t="n">
-        <v>46219</v>
-      </c>
-      <c r="R3" t="n">
-        <v>1</v>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>TAUX_REALISATION_CORRECTIF/PT</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>Chef d'atelier</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>Ameliorer le taux de realisation des OT correctifs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>13183443</v>
-      </c>
-      <c r="B4" t="n">
-        <v>4002317917</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Dysfonctionnement de température HP sort</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>OR004002317917</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>SF01-PS-PS04-SECVAP</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>SECTION VAPEUR DE L'ATELIER PS 4</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>SF1-RPS4</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>GM4</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>SF01</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>LANC CCRP PART RIMP</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>SOPL</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>BENMOUSSA1</t>
-        </is>
-      </c>
-      <c r="P4" s="2" t="n">
-        <v>46223</v>
-      </c>
-      <c r="Q4" s="2" t="n">
-        <v>46219</v>
-      </c>
-      <c r="R4" t="n">
-        <v>1</v>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>TAUX_REALISATION_CORRECTIF/PT</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>Chef d'atelier</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>Ameliorer le taux de realisation des OT correctifs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>13183444</v>
-      </c>
-      <c r="B5" t="n">
-        <v>4002317919</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Difficulté de manipulation à distance de</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>OR004002317919</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>SF01-PS-PS04-SECAIR-0K8301</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>SOUFFLANTE PRINCIPALE</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>SF1-RPS4</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>GM4</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>SF01</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>LANC CCRP PART RIMP</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>SOPL</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>BENMOUSSA1</t>
-        </is>
-      </c>
-      <c r="P5" s="2" t="n">
-        <v>46224</v>
-      </c>
-      <c r="Q5" s="2" t="n">
-        <v>46219</v>
-      </c>
-      <c r="R5" t="n">
-        <v>1</v>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>TAUX_REALISATION_CORRECTIF/PT</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>Chef d'atelier</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>Ameliorer le taux de realisation des OT correctifs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>13183445</v>
-      </c>
-      <c r="B6" t="n">
-        <v>4002317960</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>défaillance de température N° 1 du four</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>OR004002317960</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>SF01-PS-PS04-SECGAZ-0F8302</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>FOUR A COMBUSTION F8302</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>SF1-RPS4</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>GM4</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>SF01</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>LANC CCRP PART RIMP</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>SOPL</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>BENMOUSSA1</t>
-        </is>
-      </c>
-      <c r="P6" s="2" t="n">
-        <v>46224</v>
-      </c>
-      <c r="Q6" s="2" t="n">
-        <v>46219</v>
-      </c>
-      <c r="R6" t="n">
-        <v>1</v>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>TAUX_REALISATION_CORRECTIF/PT</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>Chef d'atelier</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>Ameliorer le taux de realisation des OT correctifs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>13264855</v>
-      </c>
-      <c r="B7" t="n">
-        <v>4002409639</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Contrôle et remise en état de la vanne T</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>OR004002409639</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>SF01-PS-PS04-SECVAP-0E8327-CSUR</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>CONTRÔLE ET SURVEILLANCE</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>SF1-RPS4</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>GM0</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>SF01</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>CRÉÉ CCRP PART</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>SOPL</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>MOUSSAHIF</t>
-        </is>
-      </c>
-      <c r="P7" s="2" t="n">
-        <v>46231</v>
-      </c>
-      <c r="Q7" s="2" t="n">
-        <v>46231</v>
-      </c>
-      <c r="R7" t="n">
-        <v>1</v>
-      </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>TAUX_REALISATION_CORRECTIF/PT</t>
-        </is>
-      </c>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>Chef d'atelier</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>Ameliorer le taux de realisation des OT correctifs.</t>
         </is>
       </c>
     </row>

</xml_diff>